<commit_message>
spreadsheets g7 and 6
</commit_message>
<xml_diff>
--- a/03. ICT 6-10/Grade 7/Unit 2 - Advanced spreadsheets_/Lesson 1/Worksheet - 4.1_2_3_4_5 activities.xlsx
+++ b/03. ICT 6-10/Grade 7/Unit 2 - Advanced spreadsheets_/Lesson 1/Worksheet - 4.1_2_3_4_5 activities.xlsx
@@ -1,155 +1,160 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Activity 4.1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Activity 4.2" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Activity 4.3" sheetId="3" r:id="rId7"/>
-    <sheet state="visible" name="Activity 4.4" sheetId="4" r:id="rId8"/>
-    <sheet state="visible" name="Activity 4.5" sheetId="5" r:id="rId9"/>
+    <sheet name="Activity 4.1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Activity 4.2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Activity 4.3" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Activity 4.4" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Activity 4.5" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
-    <t>Activity 4.4: Stock levels</t>
+    <t xml:space="preserve">Activity 4.1: Competition</t>
   </si>
   <si>
-    <t>Activity 4.2: Maths sets</t>
+    <t xml:space="preserve">Students have taken part in the first two rounds of a competition. To qualify for the final, they need to have scored more than 75 in both of the first two rounds.</t>
   </si>
   <si>
-    <t>Activity 4.3: Competition 2</t>
+    <t xml:space="preserve">Write a function in cell D9 to work out whether Adam has qualified for the final. It should  say "Yes" if he has qualified and "No" if he has not qualified.</t>
   </si>
   <si>
-    <t>Activity 4.1: Competition</t>
+    <t xml:space="preserve">Replicate this down to cell D13 to see if the other students have qualified for the final.</t>
   </si>
   <si>
-    <t>Students are put into sets for their maths lessons based on the mark they scored in their last exam.</t>
+    <t>Name</t>
   </si>
   <si>
-    <t>Students have taken part in the first two rounds of a competition. To qualify for the final, they need to have scored more than 75 in both of the first two rounds.</t>
+    <t xml:space="preserve">Round 1</t>
   </si>
   <si>
-    <t>A small shop uses a spreadsheet to keep track of stock levels.</t>
+    <t xml:space="preserve">Round 2</t>
   </si>
   <si>
-    <t>The rules of the competition have changed. Students now qualify for the final if they have scored more than 75 in at least one of the rounds.</t>
+    <t>Qualified?</t>
   </si>
   <si>
-    <t>For each item, if the quantity in stock is less than the re-order level or if there is a note to say that the item is 'Selling fast', then more stock needs to be ordered.</t>
+    <t>Adam</t>
   </si>
   <si>
-    <t>If they scored 75 or more they, will be put into set 1.</t>
+    <t>Bhuvan</t>
   </si>
   <si>
-    <t>If they scored less than 75 but more than 64, they will be put into set 2.</t>
+    <t>Chloe</t>
   </si>
   <si>
-    <t>If they scored less than 65, they will be put into set 3.</t>
+    <t>Devanshi</t>
   </si>
   <si>
-    <t>Write a function in cell D9 to work out whether Adam has qualified for the final. It should  say "Yes" if he has qualified and "No" if he has not qualified.</t>
+    <t>Eashan</t>
   </si>
   <si>
-    <t>Write a function in column E to show whether more stock needs to be ordered. Cells E9 to E14 should show "Yes" if more stock needs to be ordered.</t>
+    <t xml:space="preserve">Activity 4.2: Maths sets</t>
   </si>
   <si>
-    <t>Replicate this down to cell D13 to see if the other students have qualified for the final.</t>
+    <t xml:space="preserve">Students are put into sets for their maths lessons based on the mark they scored in their last exam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If they scored 75 or more they, will be put into set 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If they scored less than 75 but more than 64, they will be put into set 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If they scored less than 65, they will be put into set 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write a function in cell C12 to say "Set 2" if Adam should be put into set 2. The cell should remain empty if Adam should go into a different set.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replicate this down to cell C16 to see if the other students should be put into set 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exam %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maths set</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activity 4.3: Competition 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The rules of the competition have changed. Students now qualify for the final if they have scored more than 75 in at least one of the rounds.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activity 4.4: Stock levels</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A small shop uses a spreadsheet to keep track of stock levels.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For each item, if the quantity in stock is less than the re-order level or if there is a note to say that the item is 'Selling fast', then more stock needs to be ordered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Write a function in column E to show whether more stock needs to be ordered. Cells E9 to E14 should show "Yes" if more stock needs to be ordered.</t>
   </si>
   <si>
     <t>Item</t>
   </si>
   <si>
-    <t>Write a function in cell C12 to say "Set 2" if Adam should be put into set 2. The cell should remain empty if Adam should go into a different set.</t>
+    <t xml:space="preserve">Quantity in stock</t>
   </si>
   <si>
-    <t>Quantity in stock</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Re-order level</t>
+    <t xml:space="preserve">Re-order level</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
-    <t>Round 1</t>
-  </si>
-  <si>
-    <t>Order stock?</t>
-  </si>
-  <si>
-    <t>Round 2</t>
-  </si>
-  <si>
-    <t>Qualified?</t>
+    <t xml:space="preserve">Order stock?</t>
   </si>
   <si>
     <t>Apples</t>
   </si>
   <si>
-    <t>Replicate this down to cell C16 to see if the other students should be put into set 2.</t>
-  </si>
-  <si>
-    <t>Exam %</t>
-  </si>
-  <si>
-    <t>Adam</t>
-  </si>
-  <si>
-    <t>Maths set</t>
-  </si>
-  <si>
     <t>Oranges</t>
-  </si>
-  <si>
-    <t>Bhuvan</t>
   </si>
   <si>
     <t>Pears</t>
   </si>
   <si>
-    <t>Chloe</t>
-  </si>
-  <si>
     <t>Bananas</t>
   </si>
   <si>
-    <t>Selling fast</t>
+    <t xml:space="preserve">Selling fast</t>
   </si>
   <si>
     <t>Peaches</t>
   </si>
   <si>
-    <t>Devanshi</t>
-  </si>
-  <si>
     <t>Strawberries</t>
   </si>
   <si>
-    <t>Eashan</t>
+    <t xml:space="preserve">Activity 4.5: Homework</t>
   </si>
   <si>
-    <t>Activity 4.5: Homework</t>
+    <t xml:space="preserve">This spreadsheet shows whether students handed their homework in on time. 'G' means that it was on time and 'L' means that it was late.</t>
   </si>
   <si>
-    <t>This spreadsheet shows whether students handed their homework in on time. 'G' means that it was on time and 'L' means that it was late.</t>
+    <t xml:space="preserve">Write a function in cell H10 to count how many pieces of homework Adam handed in late. Then replicate the function down to cell H14.</t>
   </si>
   <si>
-    <t>Write a function in cell H10 to count how many pieces of homework Adam handed in late. Then replicate the function down to cell H14.</t>
+    <t xml:space="preserve">Write a function in cell I10 so that each piece of homework Adam handed in late is represented by an 'N'. Replicate the function down to cell I14.</t>
   </si>
   <si>
-    <t>Write a function in cell I10 so that each piece of homework Adam handed in late is represented by an 'X'. Replicate the function down to cell I14.</t>
-  </si>
-  <si>
-    <t>If students have handed in their Maths, English and Science homework late they are given a detention. Write a function in cell J10 to show 'Yes' if Adam has a detention. Then replicate this function down to cell J14.</t>
+    <t xml:space="preserve">If students have handed in their Maths, English and Science homework late they are given a detention. Write a function in cell J10 to show 'Yes' if Adam has a detention. Then replicate this function down to cell J14.</t>
   </si>
   <si>
     <t>Computing</t>
@@ -170,10 +175,10 @@
     <t>Science</t>
   </si>
   <si>
-    <t>Number handed in late</t>
+    <t xml:space="preserve">Number handed in late</t>
   </si>
   <si>
-    <t>X</t>
+    <t>N</t>
   </si>
   <si>
     <t>Detention</t>
@@ -188,48 +193,48 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="8">
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="20.0"/>
-      <color rgb="FF000000"/>
+      <sz val="20.000000"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color rgb="FFC55A11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
-      <color rgb="FF000000"/>
+      <sz val="14.000000"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="14.0"/>
+      <sz val="14.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="14.0"/>
-      <color rgb="FF000000"/>
+      <sz val="14.000000"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="14.0"/>
+      <sz val="14.000000"/>
       <color theme="1"/>
       <name val="Calibri"/>
     </font>
@@ -239,96 +244,368 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="19">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -385,7 +662,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -411,7 +688,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -488,7 +765,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -518,25 +795,27 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="12.67"/>
-    <col customWidth="1" min="2" max="3" width="11.0"/>
-    <col customWidth="1" min="4" max="4" width="11.33"/>
-    <col customWidth="1" min="5" max="24" width="11.0"/>
+    <col customWidth="1" min="2" max="3" width="11"/>
+    <col customWidth="1" min="4" max="4" width="16.25390625"/>
+    <col customWidth="1" min="5" max="24" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="45.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
@@ -557,294 +836,294 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
+        <v>1</v>
+      </c>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
+      <c r="A8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="8"/>
+      <c r="Z8" s="8"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="10">
-        <v>71.0</v>
-      </c>
-      <c r="C9" s="10">
-        <v>74.0</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
+      <c r="A9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9">
+        <v>71</v>
+      </c>
+      <c r="C9" s="9">
+        <v>74</v>
+      </c>
+      <c r="D9" s="10"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+      <c r="Z9" s="8"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="10">
-        <v>63.0</v>
-      </c>
-      <c r="C10" s="10">
-        <v>76.0</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="9"/>
+      <c r="A10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9">
+        <v>63</v>
+      </c>
+      <c r="C10" s="9">
+        <v>76</v>
+      </c>
+      <c r="D10" s="10"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="8"/>
+      <c r="Z10" s="8"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="10">
-        <v>73.0</v>
-      </c>
-      <c r="C11" s="10">
-        <v>75.0</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
+      <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9">
+        <v>73</v>
+      </c>
+      <c r="C11" s="9">
+        <v>75</v>
+      </c>
+      <c r="D11" s="10"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+      <c r="Z11" s="8"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="10">
-        <v>82.0</v>
-      </c>
-      <c r="C12" s="10">
-        <v>77.0</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
+      <c r="A12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9">
+        <v>82</v>
+      </c>
+      <c r="C12" s="9">
+        <v>77</v>
+      </c>
+      <c r="D12" s="10"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="10">
-        <v>78.0</v>
-      </c>
-      <c r="C13" s="10">
-        <v>81.0</v>
-      </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
+      <c r="A13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9">
+        <v>78</v>
+      </c>
+      <c r="C13" s="9">
+        <v>81</v>
+      </c>
+      <c r="D13" s="10"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="D14" s="2"/>
@@ -2254,28 +2533,29 @@
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A6:M6"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="12.11"/>
-    <col customWidth="1" min="2" max="3" width="10.78"/>
-    <col customWidth="1" min="4" max="23" width="11.0"/>
+    <col customWidth="1" min="1" max="1" width="12.109999999999999"/>
+    <col customWidth="1" min="2" max="3" width="10.779999999999999"/>
+    <col customWidth="1" min="4" max="23" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="39" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
@@ -2297,337 +2577,337 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
+        <v>14</v>
+      </c>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
-      <c r="Z4" s="4"/>
+      <c r="A4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="X4" s="11"/>
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="11"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="4"/>
-      <c r="S5" s="4"/>
-      <c r="T5" s="4"/>
-      <c r="U5" s="4"/>
-      <c r="V5" s="4"/>
-      <c r="W5" s="4"/>
-      <c r="X5" s="4"/>
-      <c r="Y5" s="4"/>
-      <c r="Z5" s="4"/>
+      <c r="A5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="4"/>
-      <c r="S6" s="4"/>
-      <c r="T6" s="4"/>
-      <c r="U6" s="4"/>
-      <c r="V6" s="4"/>
-      <c r="W6" s="4"/>
-      <c r="X6" s="4"/>
-      <c r="Y6" s="4"/>
-      <c r="Z6" s="4"/>
+      <c r="A6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="N6" s="11"/>
+      <c r="O6" s="11"/>
+      <c r="P6" s="11"/>
+      <c r="Q6" s="11"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="11"/>
+      <c r="T6" s="11"/>
+      <c r="U6" s="11"/>
+      <c r="V6" s="11"/>
+      <c r="W6" s="11"/>
+      <c r="X6" s="11"/>
+      <c r="Y6" s="11"/>
+      <c r="Z6" s="11"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-      <c r="L7" s="5"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
-      <c r="P7" s="5"/>
-      <c r="Q7" s="5"/>
-      <c r="R7" s="5"/>
-      <c r="S7" s="5"/>
-      <c r="T7" s="5"/>
-      <c r="U7" s="5"/>
-      <c r="V7" s="5"/>
-      <c r="W7" s="5"/>
-      <c r="X7" s="5"/>
-      <c r="Y7" s="5"/>
-      <c r="Z7" s="5"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+      <c r="R7" s="4"/>
+      <c r="S7" s="4"/>
+      <c r="T7" s="4"/>
+      <c r="U7" s="4"/>
+      <c r="V7" s="4"/>
+      <c r="W7" s="4"/>
+      <c r="X7" s="4"/>
+      <c r="Y7" s="4"/>
+      <c r="Z7" s="4"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
-      <c r="P8" s="5"/>
-      <c r="Q8" s="5"/>
-      <c r="R8" s="5"/>
-      <c r="S8" s="5"/>
-      <c r="T8" s="5"/>
-      <c r="U8" s="5"/>
-      <c r="V8" s="5"/>
-      <c r="W8" s="5"/>
-      <c r="X8" s="5"/>
-      <c r="Y8" s="5"/>
-      <c r="Z8" s="5"/>
+      <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="N8" s="4"/>
+      <c r="O8" s="4"/>
+      <c r="P8" s="4"/>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="4"/>
+      <c r="S8" s="4"/>
+      <c r="T8" s="4"/>
+      <c r="U8" s="4"/>
+      <c r="V8" s="4"/>
+      <c r="W8" s="4"/>
+      <c r="X8" s="4"/>
+      <c r="Y8" s="4"/>
+      <c r="Z8" s="4"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
-      <c r="P9" s="5"/>
-      <c r="Q9" s="5"/>
-      <c r="R9" s="5"/>
-      <c r="S9" s="5"/>
-      <c r="T9" s="5"/>
-      <c r="U9" s="5"/>
-      <c r="V9" s="5"/>
-      <c r="W9" s="5"/>
-      <c r="X9" s="5"/>
-      <c r="Y9" s="5"/>
-      <c r="Z9" s="5"/>
+      <c r="A9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="4"/>
+      <c r="Q9" s="4"/>
+      <c r="R9" s="4"/>
+      <c r="S9" s="4"/>
+      <c r="T9" s="4"/>
+      <c r="U9" s="4"/>
+      <c r="V9" s="4"/>
+      <c r="W9" s="4"/>
+      <c r="X9" s="4"/>
+      <c r="Y9" s="4"/>
+      <c r="Z9" s="4"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>27</v>
+      <c r="A11" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
+        <v>21</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+      <c r="Z11" s="8"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="10">
-        <v>71.0</v>
-      </c>
-      <c r="C12" s="11"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
+      <c r="A12" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="9">
+        <v>71</v>
+      </c>
+      <c r="C12" s="13"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B13" s="10">
-        <v>63.0</v>
-      </c>
-      <c r="C13" s="11"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
+      <c r="A13" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9">
+        <v>63</v>
+      </c>
+      <c r="C13" s="13"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B14" s="10">
-        <v>73.0</v>
-      </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="9"/>
-      <c r="Z14" s="9"/>
+      <c r="A14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="9">
+        <v>73</v>
+      </c>
+      <c r="C14" s="13"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+      <c r="Z14" s="8"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="10">
-        <v>82.0</v>
-      </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
-      <c r="Y15" s="9"/>
-      <c r="Z15" s="9"/>
+      <c r="A15" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="9">
+        <v>82</v>
+      </c>
+      <c r="C15" s="13"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+      <c r="V15" s="8"/>
+      <c r="W15" s="8"/>
+      <c r="X15" s="8"/>
+      <c r="Y15" s="8"/>
+      <c r="Z15" s="8"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B16" s="10">
-        <v>78.0</v>
-      </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="9"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="9"/>
-      <c r="T16" s="9"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
-      <c r="W16" s="9"/>
-      <c r="X16" s="9"/>
-      <c r="Y16" s="9"/>
-      <c r="Z16" s="9"/>
+      <c r="A16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="9">
+        <v>78</v>
+      </c>
+      <c r="C16" s="13"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+      <c r="V16" s="8"/>
+      <c r="W16" s="8"/>
+      <c r="X16" s="8"/>
+      <c r="Y16" s="8"/>
+      <c r="Z16" s="8"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="B17" s="2"/>
@@ -4235,28 +4515,29 @@
     <mergeCell ref="A8:M8"/>
     <mergeCell ref="A9:M9"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="3" width="11.0"/>
-    <col customWidth="1" min="4" max="4" width="10.78"/>
-    <col customWidth="1" min="5" max="24" width="11.0"/>
+    <col customWidth="1" min="1" max="3" width="11"/>
+    <col customWidth="1" min="4" max="4" width="10.779999999999999"/>
+    <col customWidth="1" min="5" max="24" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="37.5" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
@@ -4277,294 +4558,294 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
+        <v>23</v>
+      </c>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="6"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
+      <c r="A6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="D7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="9"/>
-      <c r="P8" s="9"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="9"/>
-      <c r="T8" s="9"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="9"/>
+      <c r="A8" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="8"/>
+      <c r="Z8" s="8"/>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="10">
-        <v>71.0</v>
-      </c>
-      <c r="C9" s="10">
-        <v>74.0</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
+      <c r="A9" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9">
+        <v>71</v>
+      </c>
+      <c r="C9" s="9">
+        <v>74</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+      <c r="Z9" s="8"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="10">
-        <v>63.0</v>
-      </c>
-      <c r="C10" s="10">
-        <v>76.0</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="9"/>
+      <c r="A10" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9">
+        <v>63</v>
+      </c>
+      <c r="C10" s="9">
+        <v>76</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="8"/>
+      <c r="Z10" s="8"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="10">
-        <v>73.0</v>
-      </c>
-      <c r="C11" s="10">
-        <v>75.0</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
+      <c r="A11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9">
+        <v>73</v>
+      </c>
+      <c r="C11" s="9">
+        <v>75</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+      <c r="Z11" s="8"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B12" s="10">
-        <v>82.0</v>
-      </c>
-      <c r="C12" s="10">
-        <v>77.0</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
+      <c r="A12" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="9">
+        <v>82</v>
+      </c>
+      <c r="C12" s="9">
+        <v>77</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="10">
-        <v>78.0</v>
-      </c>
-      <c r="C13" s="10">
-        <v>81.0</v>
-      </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
+      <c r="A13" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9">
+        <v>78</v>
+      </c>
+      <c r="C13" s="9">
+        <v>81</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="D14" s="2"/>
@@ -5974,31 +6255,32 @@
     <mergeCell ref="A5:M5"/>
     <mergeCell ref="A6:M6"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.11"/>
-    <col customWidth="1" min="2" max="2" width="17.67"/>
-    <col customWidth="1" min="3" max="3" width="14.78"/>
+    <col customWidth="1" min="1" max="1" width="13.109999999999999"/>
+    <col customWidth="1" min="2" max="2" width="17.670000000000002"/>
+    <col customWidth="1" min="3" max="3" width="14.779999999999999"/>
     <col customWidth="1" min="4" max="4" width="11.44"/>
-    <col customWidth="1" min="5" max="5" width="13.78"/>
-    <col customWidth="1" min="6" max="25" width="11.0"/>
+    <col customWidth="1" min="5" max="5" width="13.779999999999999"/>
+    <col customWidth="1" min="6" max="25" width="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
@@ -6022,85 +6304,85 @@
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4"/>
-      <c r="Q3" s="4"/>
-      <c r="R3" s="4"/>
-      <c r="S3" s="4"/>
-      <c r="T3" s="4"/>
-      <c r="U3" s="4"/>
-      <c r="V3" s="4"/>
-      <c r="W3" s="4"/>
-      <c r="X3" s="4"/>
-      <c r="Y3" s="4"/>
-      <c r="Z3" s="4"/>
+        <v>25</v>
+      </c>
+      <c r="N3" s="11"/>
+      <c r="O3" s="11"/>
+      <c r="P3" s="11"/>
+      <c r="Q3" s="11"/>
+      <c r="R3" s="11"/>
+      <c r="S3" s="11"/>
+      <c r="T3" s="11"/>
+      <c r="U3" s="11"/>
+      <c r="V3" s="11"/>
+      <c r="W3" s="11"/>
+      <c r="X3" s="11"/>
+      <c r="Y3" s="11"/>
+      <c r="Z3" s="11"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="4"/>
-      <c r="S4" s="4"/>
-      <c r="T4" s="4"/>
-      <c r="U4" s="4"/>
-      <c r="V4" s="4"/>
-      <c r="W4" s="4"/>
-      <c r="X4" s="4"/>
-      <c r="Y4" s="4"/>
-      <c r="Z4" s="4"/>
+      <c r="A4" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
+      <c r="U4" s="11"/>
+      <c r="V4" s="11"/>
+      <c r="W4" s="11"/>
+      <c r="X4" s="11"/>
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="11"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="4"/>
+      <c r="K5" s="4"/>
+      <c r="L5" s="4"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="N6" s="5"/>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5"/>
-      <c r="Q6" s="5"/>
-      <c r="R6" s="5"/>
-      <c r="S6" s="5"/>
-      <c r="T6" s="5"/>
-      <c r="U6" s="5"/>
-      <c r="V6" s="5"/>
-      <c r="W6" s="5"/>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5"/>
-      <c r="Z6" s="5"/>
+      <c r="A6" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" s="4"/>
+      <c r="O6" s="4"/>
+      <c r="P6" s="4"/>
+      <c r="Q6" s="4"/>
+      <c r="R6" s="4"/>
+      <c r="S6" s="4"/>
+      <c r="T6" s="4"/>
+      <c r="U6" s="4"/>
+      <c r="V6" s="4"/>
+      <c r="W6" s="4"/>
+      <c r="X6" s="4"/>
+      <c r="Y6" s="4"/>
+      <c r="Z6" s="4"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="B7" s="2"/>
@@ -6109,229 +6391,229 @@
       <c r="E7" s="2"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>22</v>
+      <c r="A8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B9" s="10">
-        <v>97.0</v>
-      </c>
-      <c r="C9" s="10">
-        <v>100.0</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="9"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="9"/>
-      <c r="T9" s="9"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="9"/>
+      <c r="A9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="9">
+        <v>97</v>
+      </c>
+      <c r="C9" s="9">
+        <v>100</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+      <c r="Z9" s="8"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="9">
+        <v>83</v>
+      </c>
+      <c r="C10" s="9">
+        <v>50</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="8"/>
+      <c r="Z10" s="8"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="9">
+        <v>29</v>
+      </c>
+      <c r="C11" s="9">
         <v>30</v>
       </c>
-      <c r="B10" s="10">
-        <v>83.0</v>
-      </c>
-      <c r="C10" s="10">
-        <v>50.0</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="9"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="10">
-        <v>29.0</v>
-      </c>
-      <c r="C11" s="10">
-        <v>30.0</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+      <c r="Z11" s="8"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="10">
-        <v>111.0</v>
-      </c>
-      <c r="C12" s="10">
-        <v>100.0</v>
-      </c>
-      <c r="D12" s="11" t="s">
+      <c r="A12" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="9">
+        <v>111</v>
+      </c>
+      <c r="C12" s="9">
+        <v>100</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="13"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="9">
+        <v>56</v>
+      </c>
+      <c r="C13" s="9">
+        <v>30</v>
+      </c>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="9">
+        <v>30</v>
+      </c>
+      <c r="C14" s="9">
         <v>35</v>
       </c>
-      <c r="E12" s="11"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="10">
-        <v>56.0</v>
-      </c>
-      <c r="C13" s="10">
-        <v>30.0</v>
-      </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="10">
-        <v>30.0</v>
-      </c>
-      <c r="C14" s="10">
-        <v>35.0</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="11"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="9"/>
-      <c r="Z14" s="9"/>
+      <c r="D14" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="13"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+      <c r="Z14" s="8"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="B15" s="2"/>
@@ -8356,31 +8638,32 @@
     <mergeCell ref="A4:M4"/>
     <mergeCell ref="A6:M6"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="11.22" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="11.220000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="11.11"/>
-    <col customWidth="1" min="2" max="2" width="12.0"/>
-    <col customWidth="1" min="3" max="5" width="10.78"/>
-    <col customWidth="1" min="6" max="6" width="12.11"/>
-    <col customWidth="1" min="7" max="7" width="10.78"/>
-    <col customWidth="1" min="8" max="8" width="15.78"/>
-    <col customWidth="1" min="9" max="10" width="10.78"/>
-    <col customWidth="1" min="11" max="26" width="11.0"/>
+    <col customWidth="1" min="1" max="1" width="11.109999999999999"/>
+    <col customWidth="1" min="2" max="2" width="12"/>
+    <col customWidth="1" min="3" max="5" width="10.779999999999999"/>
+    <col customWidth="1" min="6" max="6" width="12.109999999999999"/>
+    <col customWidth="1" min="7" max="7" width="10.779999999999999"/>
+    <col customWidth="1" min="8" max="8" width="15.779999999999999"/>
+    <col customWidth="1" min="9" max="10" width="10.779999999999999"/>
+    <col customWidth="1" min="11" max="26" width="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1">
+    <row r="1" ht="44.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>40</v>
       </c>
@@ -8414,105 +8697,105 @@
       <c r="A3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="4"/>
+      <c r="V3" s="4"/>
+      <c r="W3" s="4"/>
+      <c r="X3" s="4"/>
+      <c r="Y3" s="4"/>
+      <c r="Z3" s="4"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
-      <c r="K4" s="6"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="4"/>
+      <c r="N4" s="4"/>
+      <c r="O4" s="4"/>
+      <c r="P4" s="4"/>
+      <c r="Q4" s="4"/>
+      <c r="R4" s="4"/>
+      <c r="S4" s="4"/>
+      <c r="T4" s="4"/>
+      <c r="U4" s="4"/>
+      <c r="V4" s="4"/>
+      <c r="W4" s="4"/>
+      <c r="X4" s="4"/>
+      <c r="Y4" s="4"/>
+      <c r="Z4" s="4"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+      <c r="Z5" s="4"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="13"/>
-      <c r="Z6" s="13"/>
+      <c r="M6" s="14"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="14"/>
+      <c r="P6" s="14"/>
+      <c r="Q6" s="14"/>
+      <c r="R6" s="14"/>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
+      <c r="U6" s="14"/>
+      <c r="V6" s="14"/>
+      <c r="W6" s="14"/>
+      <c r="X6" s="14"/>
+      <c r="Y6" s="14"/>
+      <c r="Z6" s="14"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="13"/>
-      <c r="Z7" s="13"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="14"/>
+      <c r="O7" s="14"/>
+      <c r="P7" s="14"/>
+      <c r="Q7" s="14"/>
+      <c r="R7" s="14"/>
+      <c r="S7" s="14"/>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14"/>
+      <c r="V7" s="14"/>
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14"/>
+      <c r="Z7" s="14"/>
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="B8" s="2"/>
@@ -8525,272 +8808,272 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="15" t="s">
+    <row r="9" ht="42.75" customHeight="1">
+      <c r="A9" s="16" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="15" t="s">
+      <c r="E9" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="15" t="s">
+      <c r="G9" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="J9" s="15" t="s">
+      <c r="J9" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="17"/>
-      <c r="R9" s="17"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="17"/>
-      <c r="U9" s="17"/>
-      <c r="V9" s="17"/>
-      <c r="W9" s="17"/>
-      <c r="X9" s="17"/>
-      <c r="Y9" s="17"/>
-      <c r="Z9" s="17"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="18"/>
+      <c r="X9" s="18"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="11" t="s">
+      <c r="A10" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="9"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="9"/>
-      <c r="T10" s="9"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="9"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="8"/>
+      <c r="Z10" s="8"/>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B11" s="11" t="s">
+      <c r="A11" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F11" s="11" t="s">
+      <c r="F11" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="9"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="9"/>
-      <c r="T11" s="9"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="9"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+      <c r="Z11" s="8"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" s="11" t="s">
+      <c r="A12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="D12" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F12" s="11" t="s">
+      <c r="F12" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="G12" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="H12" s="11"/>
-      <c r="I12" s="11"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="9"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="9"/>
-      <c r="T12" s="9"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="9"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="11" t="s">
+      <c r="A13" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="F13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="G13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="9"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="9"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="11" t="s">
+      <c r="A14" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="D14" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="11" t="s">
+      <c r="F14" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="G14" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="H14" s="11"/>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="9"/>
-      <c r="Z14" s="9"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+      <c r="Z14" s="8"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="9"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -11838,9 +12121,9 @@
     <mergeCell ref="A6:L6"/>
     <mergeCell ref="A7:L7"/>
   </mergeCells>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>